<commit_message>
Cierre final del proyecto: actualización general, README y requirements y  dashboard de Power BI actualizado
</commit_message>
<xml_diff>
--- a/extras/VAN_RetailIQ360.xlsx
+++ b/extras/VAN_RetailIQ360.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\integrador_carrera\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65C80C9-ED6E-4EB7-9DED-9A247FCD7A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F29512-051A-45B1-97BD-124EC3191A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VAN " sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'VAN '!$A$1:$H$57</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'VAN '!$A$1:$H$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>RetailIQ 360° — Análisis de Valor Actual Neto (VAN)</t>
   </si>
@@ -91,12 +91,6 @@
   </si>
   <si>
     <t>Horas de análisis ad-hoc para clientes existentes. Aplica a partir del Año 2 cuando hay base instalada</t>
-  </si>
-  <si>
-    <t>Valor del activo intangible generado (plataforma)</t>
-  </si>
-  <si>
-    <t>Valorización estimada del producto a medida que se valida comercialmente. No es flujo de caja — es valor patrimonial del negocio</t>
   </si>
   <si>
     <t>Subtotal Beneficios</t>
@@ -536,131 +530,107 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -958,821 +928,804 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="37.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="11.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="89.453125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="37.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="89.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B1" s="2"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="1"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B3" s="1"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B3" s="2"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="8"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="11"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="11"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="11"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="7"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="9"/>
+    </row>
+    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="11"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="11"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="14"/>
-    </row>
-    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="10"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="15" t="s">
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="14"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H17" s="17"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H18" s="17"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="A19" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
     </row>
     <row r="21" spans="1:8" ht="26" x14ac:dyDescent="0.35">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="12" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="20"/>
-      <c r="B22" s="21" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="21" t="s">
+      <c r="E22" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="21" t="s">
+      <c r="F22" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G22" s="20"/>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-    </row>
-    <row r="24" spans="1:8" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A24" s="24" t="s">
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+    </row>
+    <row r="24" spans="1:8" s="31" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A24" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="25">
-        <v>0</v>
-      </c>
-      <c r="C24" s="25">
+      <c r="B24" s="16">
+        <v>0</v>
+      </c>
+      <c r="C24" s="16">
         <v>5400</v>
       </c>
-      <c r="D24" s="25">
-        <v>0</v>
-      </c>
-      <c r="E24" s="25">
-        <v>0</v>
-      </c>
-      <c r="F24" s="26">
-        <f t="shared" ref="F24:F28" si="0">SUM(B24:E24)</f>
+      <c r="D24" s="16">
+        <v>0</v>
+      </c>
+      <c r="E24" s="16">
+        <v>0</v>
+      </c>
+      <c r="F24" s="17">
+        <f t="shared" ref="F24:F27" si="0">SUM(B24:E24)</f>
         <v>5400</v>
       </c>
-      <c r="G24" s="27" t="s">
+      <c r="G24" s="18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A25" s="24" t="s">
+    <row r="25" spans="1:8" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A25" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="25">
-        <v>0</v>
-      </c>
-      <c r="C25" s="25">
-        <v>0</v>
-      </c>
-      <c r="D25" s="25">
+      <c r="B25" s="16">
+        <v>0</v>
+      </c>
+      <c r="C25" s="16">
+        <v>0</v>
+      </c>
+      <c r="D25" s="16">
         <f>4*400*12</f>
         <v>19200</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="16">
         <f>10*400*12</f>
         <v>48000</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="17">
         <f t="shared" si="0"/>
         <v>67200</v>
       </c>
-      <c r="G25" s="27" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A26" s="24" t="s">
+      <c r="G25" s="18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="31" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A26" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="25">
-        <v>0</v>
-      </c>
-      <c r="C26" s="25">
+      <c r="B26" s="16">
+        <v>0</v>
+      </c>
+      <c r="C26" s="16">
         <v>1500</v>
       </c>
-      <c r="D26" s="25">
+      <c r="D26" s="16">
         <f>500*4</f>
         <v>2000</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="16">
         <f>500*10</f>
         <v>5000</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="17">
         <f t="shared" si="0"/>
         <v>8500</v>
       </c>
-      <c r="G26" s="27" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A27" s="24" t="s">
+      <c r="G26" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="31" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A27" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="25">
-        <v>0</v>
-      </c>
-      <c r="C27" s="25">
-        <v>0</v>
-      </c>
-      <c r="D27" s="25">
+      <c r="B27" s="16">
+        <v>0</v>
+      </c>
+      <c r="C27" s="16">
+        <v>0</v>
+      </c>
+      <c r="D27" s="16">
         <v>1500</v>
       </c>
-      <c r="E27" s="25">
+      <c r="E27" s="16">
         <v>4000</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="17">
         <f t="shared" si="0"/>
         <v>5500</v>
       </c>
-      <c r="G27" s="27" t="s">
+      <c r="G27" s="18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A28" s="24" t="s">
+    <row r="28" spans="1:8" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A28" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="25">
-        <v>0</v>
-      </c>
-      <c r="C28" s="25">
-        <v>5000</v>
-      </c>
-      <c r="D28" s="25">
-        <v>10000</v>
-      </c>
-      <c r="E28" s="25">
-        <v>15000</v>
-      </c>
-      <c r="F28" s="26">
-        <f t="shared" si="0"/>
-        <v>30000</v>
-      </c>
-      <c r="G28" s="27" t="s">
+      <c r="B28" s="20">
+        <f>SUM(B24:B27)</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="20">
+        <f>SUM(C24:C27)</f>
+        <v>6900</v>
+      </c>
+      <c r="D28" s="20">
+        <f>SUM(D24:D27)</f>
+        <v>22700</v>
+      </c>
+      <c r="E28" s="20">
+        <f>SUM(E24:E27)</f>
+        <v>57000</v>
+      </c>
+      <c r="F28" s="20">
+        <f>SUM(F24:F27)</f>
+        <v>86600</v>
+      </c>
+      <c r="G28" s="21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A29" s="28" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+    </row>
+    <row r="30" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="B29" s="29">
-        <f>SUM(B24:B28)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="29">
-        <f>SUM(C24:C28)</f>
-        <v>11900</v>
-      </c>
-      <c r="D29" s="29">
-        <f>SUM(D24:D28)</f>
-        <v>32700</v>
-      </c>
-      <c r="E29" s="29">
-        <f>SUM(E24:E28)</f>
-        <v>72000</v>
-      </c>
-      <c r="F29" s="29">
-        <f>SUM(F24:F28)</f>
-        <v>116600</v>
-      </c>
-      <c r="G29" s="30" t="s">
+      <c r="B30" s="40"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+    </row>
+    <row r="31" spans="1:8" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A31" s="15" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="22" t="s">
+      <c r="B31" s="16">
+        <v>240</v>
+      </c>
+      <c r="C31" s="16">
+        <v>240</v>
+      </c>
+      <c r="D31" s="16">
+        <v>240</v>
+      </c>
+      <c r="E31" s="16">
+        <v>240</v>
+      </c>
+      <c r="F31" s="17">
+        <f t="shared" ref="F31:F39" si="1">SUM(B31:E31)</f>
+        <v>960</v>
+      </c>
+      <c r="G31" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-    </row>
-    <row r="32" spans="1:8" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A32" s="24" t="s">
+    </row>
+    <row r="32" spans="1:8" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A32" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="25">
+      <c r="B32" s="16">
         <v>240</v>
       </c>
-      <c r="C32" s="25">
+      <c r="C32" s="16">
         <v>240</v>
       </c>
-      <c r="D32" s="25">
+      <c r="D32" s="16">
         <v>240</v>
       </c>
-      <c r="E32" s="25">
+      <c r="E32" s="16">
         <v>240</v>
       </c>
-      <c r="F32" s="26">
-        <f t="shared" ref="F32:F40" si="1">SUM(B32:E32)</f>
-        <v>960</v>
-      </c>
-      <c r="G32" s="27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A33" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B33" s="25">
-        <v>240</v>
-      </c>
-      <c r="C33" s="25">
-        <v>240</v>
-      </c>
-      <c r="D33" s="25">
-        <v>240</v>
-      </c>
-      <c r="E33" s="25">
-        <v>240</v>
-      </c>
-      <c r="F33" s="26">
+      <c r="F32" s="17">
         <f t="shared" si="1"/>
         <v>960</v>
       </c>
-      <c r="G33" s="27" t="s">
+      <c r="G32" s="18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A33" s="15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A34" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="25">
+      <c r="B33" s="16">
         <v>120</v>
       </c>
-      <c r="C34" s="25">
+      <c r="C33" s="16">
         <v>120</v>
       </c>
-      <c r="D34" s="25">
+      <c r="D33" s="16">
         <v>120</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E33" s="16">
         <v>120</v>
       </c>
-      <c r="F34" s="26">
+      <c r="F33" s="17">
         <f t="shared" si="1"/>
         <v>480</v>
       </c>
-      <c r="G34" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A35" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B35" s="25">
-        <v>0</v>
-      </c>
-      <c r="C35" s="25">
-        <v>0</v>
-      </c>
-      <c r="D35" s="25">
+      <c r="G33" s="18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A34" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" s="16">
+        <v>0</v>
+      </c>
+      <c r="C34" s="16">
+        <v>0</v>
+      </c>
+      <c r="D34" s="16">
         <v>1200</v>
       </c>
-      <c r="E35" s="25">
+      <c r="E34" s="16">
         <v>2400</v>
       </c>
-      <c r="F35" s="26">
+      <c r="F34" s="17">
         <f t="shared" si="1"/>
         <v>3600</v>
       </c>
-      <c r="G35" s="27" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A36" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" s="25">
-        <v>0</v>
-      </c>
-      <c r="C36" s="25">
-        <v>0</v>
-      </c>
-      <c r="D36" s="25">
-        <v>0</v>
-      </c>
-      <c r="E36" s="25">
+      <c r="G34" s="18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="31" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A35" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" s="16">
+        <v>0</v>
+      </c>
+      <c r="C35" s="16">
+        <v>0</v>
+      </c>
+      <c r="D35" s="16">
+        <v>0</v>
+      </c>
+      <c r="E35" s="16">
         <v>8820</v>
       </c>
-      <c r="F36" s="26">
+      <c r="F35" s="17">
         <f t="shared" si="1"/>
         <v>8820</v>
       </c>
-      <c r="G36" s="27" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A37" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="B37" s="25">
+      <c r="G35" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A36" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="16">
         <v>360</v>
       </c>
-      <c r="C37" s="25">
+      <c r="C36" s="16">
         <v>360</v>
       </c>
-      <c r="D37" s="25">
+      <c r="D36" s="16">
         <v>360</v>
       </c>
-      <c r="E37" s="25">
+      <c r="E36" s="16">
         <v>360</v>
       </c>
-      <c r="F37" s="26">
+      <c r="F36" s="17">
         <f t="shared" si="1"/>
         <v>1440</v>
       </c>
-      <c r="G37" s="27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A38" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" s="25">
-        <v>0</v>
-      </c>
-      <c r="C38" s="25">
-        <v>0</v>
-      </c>
-      <c r="D38" s="25">
-        <v>0</v>
-      </c>
-      <c r="E38" s="25">
+      <c r="G36" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A37" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" s="16">
+        <v>0</v>
+      </c>
+      <c r="C37" s="16">
+        <v>0</v>
+      </c>
+      <c r="D37" s="16">
+        <v>0</v>
+      </c>
+      <c r="E37" s="16">
         <v>2300</v>
       </c>
-      <c r="F38" s="26">
+      <c r="F37" s="17">
         <f t="shared" si="1"/>
         <v>2300</v>
       </c>
-      <c r="G38" s="27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A39" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B39" s="25">
-        <v>0</v>
-      </c>
-      <c r="C39" s="25">
-        <v>0</v>
-      </c>
-      <c r="D39" s="25">
+      <c r="G37" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A38" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" s="16">
+        <v>0</v>
+      </c>
+      <c r="C38" s="16">
+        <v>0</v>
+      </c>
+      <c r="D38" s="16">
         <v>600</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E38" s="16">
         <v>1800</v>
       </c>
-      <c r="F39" s="26">
+      <c r="F38" s="17">
         <f t="shared" si="1"/>
         <v>2400</v>
       </c>
-      <c r="G39" s="27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" s="41" customFormat="1" ht="25" x14ac:dyDescent="0.3">
-      <c r="A40" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="B40" s="25">
+      <c r="G38" s="18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" s="31" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+      <c r="A39" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="16">
         <v>2496</v>
       </c>
-      <c r="C40" s="25">
+      <c r="C39" s="16">
         <v>2496</v>
       </c>
-      <c r="D40" s="25">
+      <c r="D39" s="16">
         <v>2496</v>
       </c>
-      <c r="E40" s="25">
+      <c r="E39" s="16">
         <v>2496</v>
       </c>
-      <c r="F40" s="26">
+      <c r="F39" s="17">
         <f t="shared" si="1"/>
         <v>9984</v>
       </c>
-      <c r="G40" s="27" t="s">
+      <c r="G39" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="31" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A40" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="23">
+        <f>SUM(B31:B39)</f>
+        <v>3456</v>
+      </c>
+      <c r="C40" s="23">
+        <f>SUM(C31:C39)</f>
+        <v>3456</v>
+      </c>
+      <c r="D40" s="23">
+        <f>SUM(D31:D39)</f>
+        <v>5256</v>
+      </c>
+      <c r="E40" s="23">
+        <f>SUM(E31:E39)</f>
+        <v>18776</v>
+      </c>
+      <c r="F40" s="23">
+        <f>SUM(F31:F39)</f>
+        <v>30944</v>
+      </c>
+      <c r="G40" s="24" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:7" s="41" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A41" s="31" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="32">
-        <f>SUM(B32:B40)</f>
-        <v>3456</v>
-      </c>
-      <c r="C41" s="32">
-        <f>SUM(C32:C40)</f>
-        <v>3456</v>
-      </c>
-      <c r="D41" s="32">
-        <f>SUM(D32:D40)</f>
-        <v>5256</v>
-      </c>
-      <c r="E41" s="32">
-        <f>SUM(E32:E40)</f>
-        <v>18776</v>
-      </c>
-      <c r="F41" s="32">
-        <f>SUM(F32:F40)</f>
-        <v>30944</v>
-      </c>
-      <c r="G41" s="33" t="s">
+      <c r="B42" s="26">
+        <f>B28-B40</f>
+        <v>-3456</v>
+      </c>
+      <c r="C42" s="26">
+        <f>C28-C40</f>
+        <v>3444</v>
+      </c>
+      <c r="D42" s="26">
+        <f>D28-D40</f>
+        <v>17444</v>
+      </c>
+      <c r="E42" s="26">
+        <f>E28-E40</f>
+        <v>38224</v>
+      </c>
+      <c r="F42" s="26">
+        <f>F28-F40</f>
+        <v>55656</v>
+      </c>
+      <c r="G42" s="27" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" s="20"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-    </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" s="34" t="s">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="13"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="35">
-        <f>B29-B41</f>
-        <v>-3456</v>
-      </c>
-      <c r="C43" s="35">
-        <f>C29-C41</f>
-        <v>8444</v>
-      </c>
-      <c r="D43" s="35">
-        <f>D29-D41</f>
-        <v>27444</v>
-      </c>
-      <c r="E43" s="35">
-        <f>E29-E41</f>
-        <v>53224</v>
-      </c>
-      <c r="F43" s="35">
-        <f>F29-F41</f>
-        <v>85656</v>
-      </c>
-      <c r="G43" s="36" t="s">
+      <c r="B45" s="28">
+        <v>0.3</v>
+      </c>
+      <c r="C45" s="25"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="25"/>
+      <c r="G45" s="25"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="25" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="20"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="20"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="20"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="20"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="34" t="s">
+      <c r="B47" s="26">
+        <f t="array" ref="B47">NPV(B45,C42:E42)+B42</f>
+        <v>26913.394629039598</v>
+      </c>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="25"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B48" s="29"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="13"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="37">
-        <v>0.3</v>
-      </c>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="34" t="s">
+      <c r="B50" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="32"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="B48" s="35">
-        <f t="array" ref="B48">NPV(B46,C43:E43)+B43</f>
-        <v>43504.200273099676</v>
-      </c>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B49" s="38"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="20"/>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20"/>
-      <c r="G50" s="20"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" s="39" t="s">
+      <c r="B51" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="B51" s="40" t="s">
-        <v>65</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="32"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="39" t="s">
+      <c r="A52" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="B52" s="40" t="s">
+      <c r="B52" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="32"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" s="39" t="s">
+      <c r="A53" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B53" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" s="39" t="s">
-        <v>51</v>
-      </c>
-      <c r="B54" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
+      <c r="B53" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="B50:G50"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="A2:G2"/>
@@ -1783,14 +1736,6 @@
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="B54:G54"/>
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A23:G23"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="B51:G51"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="B53:G53"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>